<commit_message>
EPBDS-16839 Fix round wrapping beyond the Integer range with a rounding mode and rounding whole numbers as a Float
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/RoundingAndDivision.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/RoundingAndDivision.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K104"/>
+  <dimension ref="B2:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1263,7 @@
     <row r="53" ht="43.5" customHeight="1">
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>round of a Float returns an Integer, round of a BigDecimal a BigInteger, and round of an empty value is empty. round of a whole number returns it unchanged. round(x, 0) keeps the type of x, so it also rounds numbers beyond the Integer range. roundStrict rounds the binary value as it is: the sum 0.6013 + 0.0031 is stored as 0.60439999..., so round(sum, 16) is 0.6044 but roundStrict(sum, 16) is not. UNNECESSARY works when the value already has the requested places.</t>
+          <t>round of a Float returns an Integer, round of a BigDecimal a BigInteger, and round of an empty value is empty. round of a whole number returns it unchanged, and with decimal places a Double. Beyond the Integer range round gives 2147483647 or -2147483648, with a rounding mode too, so round such numbers with round(x, 0). roundStrict rounds the binary value as it is: the sum 0.6013 + 0.0031 is stored as 0.60439999..., so round(sum, 16) is 0.6044 but roundStrict(sum, 16) is not. UNNECESSARY works when the value already has the requested places.</t>
         </is>
       </c>
     </row>
@@ -1422,343 +1422,335 @@
     <row r="68">
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EmptyWhole</t>
+          <t>BeyondIntegerRange</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; round(v)</t>
+          <t>= round(5000000000.4)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EmptyPlaces</t>
+          <t>BeyondIntegerRangeDown</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; round(v, 2)</t>
+          <t>= round(5000000000.6, DOWN)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EmptyStrict</t>
+          <t>BeyondIntegerRangePlacesDown</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; roundStrict(v, 2)</t>
+          <t>= round(5000000000.6, 0, DOWN)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>NaNToZero</t>
+          <t>LargeWholePlaces</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>= round(Double.NaN)</t>
+          <t>= round(16777217, 0)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>BinarySum</t>
+          <t>EmptyWhole</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>= round(0.6013 + 0.0031, 16) ==== 0.6044</t>
+          <t>= Double v = null; round(v)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>BinarySumStrict</t>
+          <t>EmptyPlaces</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
+          <t>= Double v = null; round(v, 2)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>StrictHundreds</t>
+          <t>EmptyStrict</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(360.989778743847, -2)</t>
+          <t>= Double v = null; roundStrict(v, 2)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>StrictToZero</t>
+          <t>NaNToZero</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(32.285, -2)</t>
+          <t>= round(Double.NaN)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>ProductPlaces</t>
+          <t>BinarySum</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>= round(0.7 * 0.75, 2)</t>
+          <t>= round(0.6013 + 0.0031, 16) ==== 0.6044</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>LongProductPlaces</t>
+          <t>BinarySumStrict</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>= round(-4.65464 * -45678.65464, 2)</t>
+          <t>= roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>HalfDownPlaces</t>
+          <t>StrictHundreds</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>= round(1.005, 2, HALF_DOWN)</t>
+          <t>= roundStrict(360.989778743847, -2)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="inlineStr">
         <is>
+          <t>StrictToZero</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>= roundStrict(32.285, -2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>ProductPlaces</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>= round(0.7 * 0.75, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>LongProductPlaces</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>= round(-4.65464 * -45678.65464, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>HalfDownPlaces</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>= round(1.005, 2, HALF_DOWN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
           <t>AlreadyExact</t>
         </is>
       </c>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="C83" s="7" t="inlineStr">
         <is>
           <t>= round(32.28, 2, UNNECESSARY)</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="B81" s="3" t="inlineStr">
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>Test RoundingEdgeCases RoundingEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C81" s="8" t="n"/>
-      <c r="D81" s="4" t="n"/>
-    </row>
-    <row r="82">
-      <c r="B82" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FloatWhole</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>round(2.5f)</t>
-        </is>
-      </c>
-      <c r="D82" s="10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FloatPlaces</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>round(32.285f, 2)</t>
-        </is>
-      </c>
-      <c r="D83" s="10" t="n">
-        <v>32.29</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$DecimalWhole</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>round((BigDecimal) 32.5)</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$DecimalWholeType</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>round((BigDecimal) 32.5).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D85" s="10" t="inlineStr">
-        <is>
-          <t>BigInteger</t>
-        </is>
-      </c>
+      <c r="C85" s="8" t="n"/>
+      <c r="D85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalHalfEven</t>
+          <t>_res_.$FloatWhole</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 2.5, HALF_EVEN)</t>
+          <t>round(2.5f)</t>
         </is>
       </c>
       <c r="D86" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalPlacesDown</t>
+          <t>_res_.$FloatPlaces</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 32.285, 2, DOWN)</t>
+          <t>round(32.285f, 2)</t>
         </is>
       </c>
       <c r="D87" s="10" t="n">
-        <v>32.28</v>
+        <v>32.29</v>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroPlaces</t>
+          <t>_res_.$DecimalWhole</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>round(2.5, 0)</t>
+          <t>round((BigDecimal) 32.5)</t>
         </is>
       </c>
       <c r="D88" s="10" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="9" t="inlineStr">
         <is>
-          <t>_res_.$WholeInput</t>
+          <t>_res_.$DecimalWholeType</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Integer v = 1000000000; round(v)</t>
-        </is>
-      </c>
-      <c r="D89" s="10" t="n">
-        <v>1000000000</v>
+          <t>round((BigDecimal) 32.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>BigInteger</t>
+        </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyWholeInput</t>
+          <t>_res_.$DecimalHalfEven</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; round(v)</t>
-        </is>
-      </c>
-      <c r="D90" s="10" t="n"/>
+          <t>round((BigDecimal) 2.5, HALF_EVEN)</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NearIntegerLimit</t>
+          <t>_res_.$DecimalPlacesDown</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>round(2147483646.5)</t>
+          <t>round((BigDecimal) 32.285, 2, DOWN)</t>
         </is>
       </c>
       <c r="D91" s="10" t="n">
-        <v>2147483647</v>
+        <v>32.28</v>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondIntegerLimit</t>
+          <t>_res_.$ZeroPlaces</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>round(2147483647.5, 0)</t>
+          <t>round(2.5, 0)</t>
         </is>
       </c>
       <c r="D92" s="10" t="n">
-        <v>2147483648</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyWhole</t>
+          <t>_res_.$WholeInput</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; round(v)</t>
-        </is>
-      </c>
-      <c r="D93" s="10" t="n"/>
+          <t>Integer v = 1000000000; round(v)</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="n">
+        <v>1000000000</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyPlaces</t>
+          <t>_res_.$EmptyWholeInput</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; round(v, 2)</t>
+          <t>Integer v = null; round(v)</t>
         </is>
       </c>
       <c r="D94" s="10" t="n"/>
@@ -1766,152 +1758,268 @@
     <row r="95">
       <c r="B95" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyStrict</t>
+          <t>_res_.$NearIntegerLimit</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; roundStrict(v, 2)</t>
-        </is>
-      </c>
-      <c r="D95" s="10" t="n"/>
+          <t>round(2147483646.5)</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="n">
+        <v>2147483647</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NaNToZero</t>
+          <t>_res_.$BeyondIntegerLimit</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>round(Double.NaN)</t>
+          <t>round(2147483647.5, 0)</t>
         </is>
       </c>
       <c r="D96" s="10" t="n">
-        <v>0</v>
+        <v>2147483648</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BinarySum</t>
+          <t>_res_.$BeyondIntegerRange</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>round(0.6013 + 0.0031, 16) ==== 0.6044</t>
-        </is>
-      </c>
-      <c r="D97" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>round(5000000000.4)</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="n">
+        <v>2147483647</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BinarySumStrict</t>
+          <t>_res_.$BeyondIntegerRangeDown</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
-        </is>
-      </c>
-      <c r="D98" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+          <t>round(5000000000.6, DOWN)</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="n">
+        <v>2147483647</v>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StrictHundreds</t>
+          <t>_res_.$BeyondIntegerRangePlacesDown</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(360.989778743847, -2)</t>
+          <t>round(5000000000.6, 0, DOWN)</t>
         </is>
       </c>
       <c r="D99" s="10" t="n">
-        <v>400</v>
+        <v>5000000000</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StrictToZero</t>
+          <t>_res_.$LargeWholePlaces</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(32.285, -2)</t>
+          <t>round(16777217, 0)</t>
         </is>
       </c>
       <c r="D100" s="10" t="n">
-        <v>0</v>
+        <v>16777217</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductPlaces</t>
+          <t>_res_.$EmptyWhole</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>round(0.7 * 0.75, 2)</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="n">
-        <v>0.53</v>
-      </c>
+          <t>Double v = null; round(v)</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="n"/>
     </row>
     <row r="102">
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LongProductPlaces</t>
+          <t>_res_.$EmptyPlaces</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>round(-4.65464 * -45678.65464, 2)</t>
-        </is>
-      </c>
-      <c r="D102" s="10" t="n">
-        <v>212617.69</v>
-      </c>
+          <t>Double v = null; round(v, 2)</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="n"/>
     </row>
     <row r="103">
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>_res_.$HalfDownPlaces</t>
+          <t>_res_.$EmptyStrict</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>round(1.005, 2, HALF_DOWN)</t>
-        </is>
-      </c>
-      <c r="D103" s="10" t="n">
-        <v>1</v>
-      </c>
+          <t>Double v = null; roundStrict(v, 2)</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="9" t="inlineStr">
         <is>
+          <t>_res_.$NaNToZero</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>round(Double.NaN)</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BinarySum</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>round(0.6013 + 0.0031, 16) ==== 0.6044</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BinarySumStrict</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$StrictHundreds</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>roundStrict(360.989778743847, -2)</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$StrictToZero</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>roundStrict(32.285, -2)</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ProductPlaces</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>round(0.7 * 0.75, 2)</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$LongProductPlaces</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>round(-4.65464 * -45678.65464, 2)</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="n">
+        <v>212617.69</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$HalfDownPlaces</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>round(1.005, 2, HALF_DOWN)</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="9" t="inlineStr">
+        <is>
           <t>_res_.$AlreadyExact</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>round(32.28, 2, UNNECESSARY)</t>
         </is>
       </c>
-      <c r="D104" s="10" t="n">
+      <c r="D112" s="10" t="n">
         <v>32.28</v>
       </c>
     </row>
@@ -1920,12 +2028,12 @@
     <mergeCell ref="B55:C55"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B45:K45"/>
+    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B31:I31"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="B85:D85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-16841 Document how round treats an empty scale or rounding mode
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/RoundingAndDivision.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/RoundingAndDivision.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K112"/>
+  <dimension ref="B2:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1260,10 +1260,10 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="53" ht="43.5" customHeight="1">
+    <row r="53" ht="57" customHeight="1">
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>round of a Float returns an Integer, round of a BigDecimal a BigInteger, and round of an empty value is empty. round of a whole number returns it unchanged, and with decimal places a Double. Beyond the Integer range round gives 2147483647 or -2147483648, with a rounding mode too, so round such numbers with round(x, 0). roundStrict rounds the binary value as it is: the sum 0.6013 + 0.0031 is stored as 0.60439999..., so round(sum, 16) is 0.6044 but roundStrict(sum, 16) is not. UNNECESSARY works when the value already has the requested places.</t>
+          <t>round of a Float returns an Integer, round of a BigDecimal a BigInteger, and round of an empty value is empty. An empty number of places counts as 0, and so does an empty rounding mode number, which makes it UP. round of a whole number returns it unchanged, and with decimal places a Double. Beyond the Integer range round gives 2147483647 or -2147483648, with a rounding mode too, so round such numbers with round(x, 0). roundStrict rounds the binary value as it is: the sum 0.6013 + 0.0031 is stored as 0.60439999..., so round(sum, 16) is 0.6044 but roundStrict(sum, 16) is not. UNNECESSARY works when the value already has the requested places.</t>
         </is>
       </c>
     </row>
@@ -1506,294 +1506,288 @@
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>NaNToZero</t>
+          <t>EmptyScale</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>= round(Double.NaN)</t>
+          <t>= Integer s = null; round(2.567, s)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>BinarySum</t>
+          <t>EmptyModeNumber</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>= round(0.6013 + 0.0031, 16) ==== 0.6044</t>
+          <t>= Integer r = null; round(2.561, 2, r)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>BinarySumStrict</t>
+          <t>NaNToZero</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
+          <t>= round(Double.NaN)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>StrictHundreds</t>
+          <t>BinarySum</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(360.989778743847, -2)</t>
+          <t>= round(0.6013 + 0.0031, 16) ==== 0.6044</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>StrictToZero</t>
+          <t>BinarySumStrict</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>= roundStrict(32.285, -2)</t>
+          <t>= roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>ProductPlaces</t>
+          <t>StrictHundreds</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>= round(0.7 * 0.75, 2)</t>
+          <t>= roundStrict(360.989778743847, -2)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>LongProductPlaces</t>
+          <t>StrictToZero</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>= round(-4.65464 * -45678.65464, 2)</t>
+          <t>= roundStrict(32.285, -2)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>HalfDownPlaces</t>
+          <t>ProductPlaces</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>= round(1.005, 2, HALF_DOWN)</t>
+          <t>= round(0.7 * 0.75, 2)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="6" t="inlineStr">
         <is>
+          <t>LongProductPlaces</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>= round(-4.65464 * -45678.65464, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>HalfDownPlaces</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>= round(1.005, 2, HALF_DOWN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="6" t="inlineStr">
+        <is>
           <t>AlreadyExact</t>
         </is>
       </c>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="C85" s="7" t="inlineStr">
         <is>
           <t>= round(32.28, 2, UNNECESSARY)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" s="3" t="inlineStr">
+    <row r="87">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>Test RoundingEdgeCases RoundingEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C85" s="8" t="n"/>
-      <c r="D85" s="4" t="n"/>
-    </row>
-    <row r="86">
-      <c r="B86" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FloatWhole</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>round(2.5f)</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FloatPlaces</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>round(32.285f, 2)</t>
-        </is>
-      </c>
-      <c r="D87" s="10" t="n">
-        <v>32.29</v>
-      </c>
+      <c r="C87" s="8" t="n"/>
+      <c r="D87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="B88" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalWhole</t>
+          <t>_res_.$FloatWhole</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 32.5)</t>
+          <t>round(2.5f)</t>
         </is>
       </c>
       <c r="D88" s="10" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalWholeType</t>
+          <t>_res_.$FloatPlaces</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 32.5).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D89" s="10" t="inlineStr">
-        <is>
-          <t>BigInteger</t>
-        </is>
+          <t>round(32.285f, 2)</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="n">
+        <v>32.29</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalHalfEven</t>
+          <t>_res_.$DecimalWhole</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 2.5, HALF_EVEN)</t>
+          <t>round((BigDecimal) 32.5)</t>
         </is>
       </c>
       <c r="D90" s="10" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DecimalPlacesDown</t>
+          <t>_res_.$DecimalWholeType</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>round((BigDecimal) 32.285, 2, DOWN)</t>
-        </is>
-      </c>
-      <c r="D91" s="10" t="n">
-        <v>32.28</v>
+          <t>round((BigDecimal) 32.5).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="inlineStr">
+        <is>
+          <t>BigInteger</t>
+        </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroPlaces</t>
+          <t>_res_.$DecimalHalfEven</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>round(2.5, 0)</t>
+          <t>round((BigDecimal) 2.5, HALF_EVEN)</t>
         </is>
       </c>
       <c r="D92" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>_res_.$WholeInput</t>
+          <t>_res_.$DecimalPlacesDown</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Integer v = 1000000000; round(v)</t>
+          <t>round((BigDecimal) 32.285, 2, DOWN)</t>
         </is>
       </c>
       <c r="D93" s="10" t="n">
-        <v>1000000000</v>
+        <v>32.28</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyWholeInput</t>
+          <t>_res_.$ZeroPlaces</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Integer v = null; round(v)</t>
-        </is>
-      </c>
-      <c r="D94" s="10" t="n"/>
+          <t>round(2.5, 0)</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NearIntegerLimit</t>
+          <t>_res_.$WholeInput</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>round(2147483646.5)</t>
+          <t>Integer v = 1000000000; round(v)</t>
         </is>
       </c>
       <c r="D95" s="10" t="n">
-        <v>2147483647</v>
+        <v>1000000000</v>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondIntegerLimit</t>
+          <t>_res_.$EmptyWholeInput</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>round(2147483647.5, 0)</t>
-        </is>
-      </c>
-      <c r="D96" s="10" t="n">
-        <v>2147483648</v>
-      </c>
+          <t>Integer v = null; round(v)</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondIntegerRange</t>
+          <t>_res_.$NearIntegerLimit</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>round(5000000000.4)</t>
+          <t>round(2147483646.5)</t>
         </is>
       </c>
       <c r="D97" s="10" t="n">
@@ -1803,83 +1797,87 @@
     <row r="98">
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondIntegerRangeDown</t>
+          <t>_res_.$BeyondIntegerLimit</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>round(5000000000.6, DOWN)</t>
+          <t>round(2147483647.5, 0)</t>
         </is>
       </c>
       <c r="D98" s="10" t="n">
-        <v>2147483647</v>
+        <v>2147483648</v>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondIntegerRangePlacesDown</t>
+          <t>_res_.$BeyondIntegerRange</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>round(5000000000.6, 0, DOWN)</t>
+          <t>round(5000000000.4)</t>
         </is>
       </c>
       <c r="D99" s="10" t="n">
-        <v>5000000000</v>
+        <v>2147483647</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LargeWholePlaces</t>
+          <t>_res_.$BeyondIntegerRangeDown</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>round(16777217, 0)</t>
+          <t>round(5000000000.6, DOWN)</t>
         </is>
       </c>
       <c r="D100" s="10" t="n">
-        <v>16777217</v>
+        <v>2147483647</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyWhole</t>
+          <t>_res_.$BeyondIntegerRangePlacesDown</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; round(v)</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="n"/>
+          <t>round(5000000000.6, 0, DOWN)</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="n">
+        <v>5000000000</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyPlaces</t>
+          <t>_res_.$LargeWholePlaces</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; round(v, 2)</t>
-        </is>
-      </c>
-      <c r="D102" s="10" t="n"/>
+          <t>round(16777217, 0)</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="n">
+        <v>16777217</v>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyStrict</t>
+          <t>_res_.$EmptyWhole</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; roundStrict(v, 2)</t>
+          <t>Double v = null; round(v)</t>
         </is>
       </c>
       <c r="D103" s="10" t="n"/>
@@ -1887,76 +1885,68 @@
     <row r="104">
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NaNToZero</t>
+          <t>_res_.$EmptyPlaces</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>round(Double.NaN)</t>
-        </is>
-      </c>
-      <c r="D104" s="10" t="n">
-        <v>0</v>
-      </c>
+          <t>Double v = null; round(v, 2)</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="n"/>
     </row>
     <row r="105">
       <c r="B105" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BinarySum</t>
+          <t>_res_.$EmptyStrict</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>round(0.6013 + 0.0031, 16) ==== 0.6044</t>
-        </is>
-      </c>
-      <c r="D105" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Double v = null; roundStrict(v, 2)</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="n"/>
     </row>
     <row r="106">
       <c r="B106" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BinarySumStrict</t>
+          <t>_res_.$EmptyScale</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
-        </is>
-      </c>
-      <c r="D106" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+          <t>Integer s = null; round(2.567, s)</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StrictHundreds</t>
+          <t>_res_.$EmptyModeNumber</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(360.989778743847, -2)</t>
+          <t>Integer r = null; round(2.561, 2, r)</t>
         </is>
       </c>
       <c r="D107" s="10" t="n">
-        <v>400</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>_res_.$StrictToZero</t>
+          <t>_res_.$NaNToZero</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>roundStrict(32.285, -2)</t>
+          <t>round(Double.NaN)</t>
         </is>
       </c>
       <c r="D108" s="10" t="n">
@@ -1966,60 +1956,124 @@
     <row r="109">
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ProductPlaces</t>
+          <t>_res_.$BinarySum</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>round(0.7 * 0.75, 2)</t>
-        </is>
-      </c>
-      <c r="D109" s="10" t="n">
-        <v>0.53</v>
+          <t>round(0.6013 + 0.0031, 16) ==== 0.6044</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LongProductPlaces</t>
+          <t>_res_.$BinarySumStrict</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>round(-4.65464 * -45678.65464, 2)</t>
-        </is>
-      </c>
-      <c r="D110" s="10" t="n">
-        <v>212617.69</v>
+          <t>roundStrict(0.6013 + 0.0031, 16) ==== 0.6044</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" s="9" t="inlineStr">
         <is>
-          <t>_res_.$HalfDownPlaces</t>
+          <t>_res_.$StrictHundreds</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>round(1.005, 2, HALF_DOWN)</t>
+          <t>roundStrict(360.989778743847, -2)</t>
         </is>
       </c>
       <c r="D111" s="10" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="9" t="inlineStr">
         <is>
+          <t>_res_.$StrictToZero</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>roundStrict(32.285, -2)</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ProductPlaces</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>round(0.7 * 0.75, 2)</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$LongProductPlaces</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>round(-4.65464 * -45678.65464, 2)</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="n">
+        <v>212617.69</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$HalfDownPlaces</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>round(1.005, 2, HALF_DOWN)</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="9" t="inlineStr">
+        <is>
           <t>_res_.$AlreadyExact</t>
         </is>
       </c>
-      <c r="C112" s="5" t="inlineStr">
+      <c r="C116" s="5" t="inlineStr">
         <is>
           <t>round(32.28, 2, UNNECESSARY)</t>
         </is>
       </c>
-      <c r="D112" s="10" t="n">
+      <c r="D116" s="10" t="n">
         <v>32.28</v>
       </c>
     </row>
@@ -2031,9 +2085,9 @@
     <mergeCell ref="B53:I53"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B87:D87"/>
     <mergeCell ref="B31:I31"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B85:D85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>